<commit_message>
Mise à jour du fichier Excel
</commit_message>
<xml_diff>
--- a/base_de_connaissance.xlsx
+++ b/base_de_connaissance.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\OneDrive\Bureau\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\AWS\projetGIT2\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E9E210-44EA-4854-889F-869C565992E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Entrées base de connaissances" sheetId="1" r:id="rId1"/>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="100">
   <si>
     <t>Problème n°</t>
   </si>
@@ -321,12 +322,66 @@
   <si>
     <t>exemple 8</t>
   </si>
+  <si>
+    <t>Ex. 9</t>
+  </si>
+  <si>
+    <t>An error occurred (InvalidAMIID.NotFound) when calling the RunInstances operation: The image id '[ami-0126145f1f70769be]' does not exist</t>
+  </si>
+  <si>
+    <t>On a script qui crée une instance EC2 automatiquement mais qui échoue</t>
+  </si>
+  <si>
+    <t>utilisation d'une region inapproprié</t>
+  </si>
+  <si>
+    <t>dans le script y'a une partie où la region est ecrite textuellement au lieu d'utiliser la variable $region directement pour eviter de faire des erreurs lors de al saisie manuelle.</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>Utiliser les variables pour stocker les informations d'un script au lieu de faire la saie manuelle chaque fois</t>
+  </si>
+  <si>
+    <t>exemple 9</t>
+  </si>
+  <si>
+    <t>173--Lab - Résolution des problèmes de création d'instance</t>
+  </si>
+  <si>
+    <t>N /A</t>
+  </si>
+  <si>
+    <t>exemple 10</t>
+  </si>
+  <si>
+    <t>Une erreur s'est produite lors de la création de trigger: Configurations overlap. Configurations on the same bucket cannot share a common event type.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'ancien trigger S3 de la première fonction existe encore. </t>
+  </si>
+  <si>
+    <t>j'avais mis node.js comme runtime de mon code python</t>
+  </si>
+  <si>
+    <t>Supprimer l'ancien trigger depuis S3</t>
+  </si>
+  <si>
+    <t>recherche google</t>
+  </si>
+  <si>
+    <t>177--Lab - [Challenge] Exercice sur AWS Lambda</t>
+  </si>
+  <si>
+    <t>EX. 10</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="16">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -428,6 +483,18 @@
       <sz val="16"/>
       <color rgb="FF3F3F76"/>
       <name val="Amazon Ember Light"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -664,7 +731,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -767,6 +834,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1082,23 +1155,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z188"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="20"/>
+  <dimension ref="A1:Z190"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="20.399999999999999"/>
   <cols>
-    <col min="1" max="1" width="28.6328125" style="2" customWidth="1"/>
-    <col min="2" max="3" width="32.453125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="81.54296875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="47.08984375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="57.36328125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="56.08984375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="73.08984375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="61.6328125" style="2" customWidth="1"/>
-    <col min="10" max="10" width="11.453125" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="11.453125" style="2"/>
+    <col min="1" max="1" width="28.6640625" style="2" customWidth="1"/>
+    <col min="2" max="3" width="32.44140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="81.5546875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="47.109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="57.33203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="56.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="73.109375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="61.6640625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="11.44140625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" s="11" customFormat="1" ht="65.400000000000006" customHeight="1" thickBot="1">
@@ -1128,7 +1201,7 @@
       </c>
       <c r="I1" s="10"/>
     </row>
-    <row r="2" spans="1:26" ht="409.25" customHeight="1">
+    <row r="2" spans="1:26" ht="409.2" customHeight="1">
       <c r="A2" s="19" t="s">
         <v>8</v>
       </c>
@@ -1428,542 +1501,634 @@
       <c r="Y9" s="34"/>
       <c r="Z9" s="34"/>
     </row>
-    <row r="10" spans="1:26" ht="22.75" customHeight="1">
-      <c r="A10" s="4"/>
-    </row>
-    <row r="11" spans="1:26" ht="22.75" customHeight="1">
-      <c r="A11" s="4"/>
-    </row>
-    <row r="12" spans="1:26" ht="22.75" customHeight="1">
+    <row r="10" spans="1:26" ht="207" customHeight="1">
+      <c r="A10" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="B10" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="C10" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="D10" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="E10" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="F10" s="32" t="s">
+        <v>86</v>
+      </c>
+      <c r="G10" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="H10" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="I10" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="J10" s="34"/>
+      <c r="K10" s="34"/>
+      <c r="L10" s="34"/>
+      <c r="M10" s="34"/>
+      <c r="N10" s="34"/>
+      <c r="O10" s="34"/>
+      <c r="P10" s="34"/>
+      <c r="Q10" s="34"/>
+      <c r="R10" s="34"/>
+      <c r="S10" s="34"/>
+      <c r="T10" s="34"/>
+      <c r="U10" s="34"/>
+      <c r="V10" s="34"/>
+      <c r="W10" s="34"/>
+      <c r="X10" s="34"/>
+      <c r="Y10" s="34"/>
+      <c r="Z10" s="34"/>
+    </row>
+    <row r="11" spans="1:26" ht="207" customHeight="1">
+      <c r="A11" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="B11" s="31" t="s">
+        <v>98</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>94</v>
+      </c>
+      <c r="D11" s="35" t="s">
+        <v>93</v>
+      </c>
+      <c r="E11" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="F11" s="36" t="s">
+        <v>96</v>
+      </c>
+      <c r="G11" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="H11" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="I11" s="33" t="s">
+        <v>92</v>
+      </c>
+      <c r="J11" s="34"/>
+      <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
+      <c r="M11" s="34"/>
+      <c r="N11" s="34"/>
+      <c r="O11" s="34"/>
+      <c r="P11" s="34"/>
+      <c r="Q11" s="34"/>
+      <c r="R11" s="34"/>
+      <c r="S11" s="34"/>
+      <c r="T11" s="34"/>
+      <c r="U11" s="34"/>
+      <c r="V11" s="34"/>
+      <c r="W11" s="34"/>
+      <c r="X11" s="34"/>
+      <c r="Y11" s="34"/>
+      <c r="Z11" s="34"/>
+    </row>
+    <row r="12" spans="1:26" ht="22.8" customHeight="1">
       <c r="A12" s="4"/>
     </row>
-    <row r="13" spans="1:26" ht="22.75" customHeight="1">
+    <row r="13" spans="1:26" ht="22.8" customHeight="1">
       <c r="A13" s="4"/>
     </row>
-    <row r="14" spans="1:26" ht="22.75" customHeight="1">
+    <row r="14" spans="1:26" ht="22.8" customHeight="1">
       <c r="A14" s="4"/>
     </row>
-    <row r="15" spans="1:26" ht="22.75" customHeight="1">
+    <row r="15" spans="1:26" ht="22.8" customHeight="1">
       <c r="A15" s="4"/>
     </row>
-    <row r="16" spans="1:26" ht="22.75" customHeight="1">
+    <row r="16" spans="1:26" ht="22.8" customHeight="1">
       <c r="A16" s="4"/>
     </row>
-    <row r="17" spans="1:1" ht="22.75" customHeight="1">
+    <row r="17" spans="1:1" ht="22.8" customHeight="1">
       <c r="A17" s="4"/>
     </row>
-    <row r="18" spans="1:1" ht="22.75" customHeight="1">
+    <row r="18" spans="1:1" ht="22.8" customHeight="1">
       <c r="A18" s="4"/>
     </row>
-    <row r="19" spans="1:1" ht="22.75" customHeight="1">
+    <row r="19" spans="1:1" ht="22.8" customHeight="1">
       <c r="A19" s="4"/>
     </row>
-    <row r="20" spans="1:1" ht="22.75" customHeight="1">
+    <row r="20" spans="1:1" ht="22.8" customHeight="1">
       <c r="A20" s="4"/>
     </row>
-    <row r="21" spans="1:1" ht="22.75" customHeight="1">
+    <row r="21" spans="1:1" ht="22.8" customHeight="1">
       <c r="A21" s="4"/>
     </row>
-    <row r="22" spans="1:1" ht="22.75" customHeight="1">
+    <row r="22" spans="1:1" ht="22.8" customHeight="1">
       <c r="A22" s="4"/>
     </row>
-    <row r="23" spans="1:1" ht="22.75" customHeight="1">
+    <row r="23" spans="1:1" ht="22.8" customHeight="1">
       <c r="A23" s="4"/>
     </row>
-    <row r="24" spans="1:1" ht="22.75" customHeight="1">
+    <row r="24" spans="1:1" ht="22.8" customHeight="1">
       <c r="A24" s="4"/>
     </row>
-    <row r="25" spans="1:1" ht="22.75" customHeight="1">
+    <row r="25" spans="1:1" ht="22.8" customHeight="1">
       <c r="A25" s="4"/>
     </row>
-    <row r="26" spans="1:1" ht="22.75" customHeight="1">
+    <row r="26" spans="1:1" ht="22.8" customHeight="1">
       <c r="A26" s="4"/>
     </row>
-    <row r="27" spans="1:1" ht="22.75" customHeight="1">
+    <row r="27" spans="1:1" ht="22.8" customHeight="1">
       <c r="A27" s="4"/>
     </row>
-    <row r="28" spans="1:1" ht="22.75" customHeight="1">
+    <row r="28" spans="1:1" ht="22.8" customHeight="1">
       <c r="A28" s="4"/>
     </row>
-    <row r="29" spans="1:1" ht="22.75" customHeight="1">
+    <row r="29" spans="1:1" ht="22.8" customHeight="1">
       <c r="A29" s="4"/>
     </row>
-    <row r="30" spans="1:1" ht="22.75" customHeight="1">
+    <row r="30" spans="1:1" ht="22.8" customHeight="1">
       <c r="A30" s="4"/>
     </row>
-    <row r="31" spans="1:1" ht="22.75" customHeight="1">
+    <row r="31" spans="1:1" ht="22.8" customHeight="1">
       <c r="A31" s="4"/>
     </row>
-    <row r="32" spans="1:1" ht="22.75" customHeight="1">
+    <row r="32" spans="1:1" ht="22.8" customHeight="1">
       <c r="A32" s="4"/>
     </row>
-    <row r="33" spans="1:1" ht="22.75" customHeight="1">
+    <row r="33" spans="1:1" ht="22.8" customHeight="1">
       <c r="A33" s="4"/>
     </row>
-    <row r="34" spans="1:1" ht="22.75" customHeight="1">
+    <row r="34" spans="1:1" ht="22.8" customHeight="1">
       <c r="A34" s="4"/>
     </row>
-    <row r="35" spans="1:1" ht="22.75" customHeight="1">
+    <row r="35" spans="1:1" ht="22.8" customHeight="1">
       <c r="A35" s="4"/>
     </row>
-    <row r="36" spans="1:1" ht="22.75" customHeight="1">
+    <row r="36" spans="1:1" ht="22.8" customHeight="1">
       <c r="A36" s="4"/>
     </row>
-    <row r="37" spans="1:1" ht="22.75" customHeight="1">
+    <row r="37" spans="1:1" ht="22.8" customHeight="1">
       <c r="A37" s="4"/>
     </row>
-    <row r="38" spans="1:1" ht="22.75" customHeight="1">
+    <row r="38" spans="1:1" ht="22.8" customHeight="1">
       <c r="A38" s="4"/>
     </row>
-    <row r="39" spans="1:1" ht="22.75" customHeight="1">
+    <row r="39" spans="1:1" ht="22.8" customHeight="1">
       <c r="A39" s="4"/>
     </row>
-    <row r="40" spans="1:1" ht="22.75" customHeight="1">
+    <row r="40" spans="1:1" ht="22.8" customHeight="1">
       <c r="A40" s="4"/>
     </row>
-    <row r="41" spans="1:1" ht="22.75" customHeight="1">
+    <row r="41" spans="1:1" ht="22.8" customHeight="1">
       <c r="A41" s="4"/>
     </row>
-    <row r="42" spans="1:1" ht="22.75" customHeight="1">
+    <row r="42" spans="1:1" ht="22.8" customHeight="1">
       <c r="A42" s="4"/>
     </row>
-    <row r="43" spans="1:1" ht="22.75" customHeight="1">
+    <row r="43" spans="1:1" ht="22.8" customHeight="1">
       <c r="A43" s="4"/>
     </row>
-    <row r="44" spans="1:1" ht="22.75" customHeight="1">
+    <row r="44" spans="1:1" ht="22.8" customHeight="1">
       <c r="A44" s="4"/>
     </row>
-    <row r="45" spans="1:1" ht="22.75" customHeight="1">
+    <row r="45" spans="1:1" ht="22.8" customHeight="1">
       <c r="A45" s="4"/>
     </row>
-    <row r="46" spans="1:1" ht="22.75" customHeight="1">
+    <row r="46" spans="1:1" ht="22.8" customHeight="1">
       <c r="A46" s="4"/>
     </row>
-    <row r="47" spans="1:1" ht="22.75" customHeight="1">
+    <row r="47" spans="1:1" ht="22.8" customHeight="1">
       <c r="A47" s="4"/>
     </row>
-    <row r="48" spans="1:1" ht="22.75" customHeight="1">
+    <row r="48" spans="1:1" ht="22.8" customHeight="1">
       <c r="A48" s="4"/>
     </row>
-    <row r="49" spans="1:1" ht="22.75" customHeight="1">
+    <row r="49" spans="1:1" ht="22.8" customHeight="1">
       <c r="A49" s="4"/>
     </row>
-    <row r="50" spans="1:1" ht="22.75" customHeight="1">
+    <row r="50" spans="1:1" ht="22.8" customHeight="1">
       <c r="A50" s="4"/>
     </row>
-    <row r="51" spans="1:1" ht="22.75" customHeight="1">
+    <row r="51" spans="1:1" ht="22.8" customHeight="1">
       <c r="A51" s="4"/>
     </row>
-    <row r="52" spans="1:1" ht="22.75" customHeight="1">
+    <row r="52" spans="1:1" ht="22.8" customHeight="1">
       <c r="A52" s="4"/>
     </row>
-    <row r="53" spans="1:1" ht="22.75" customHeight="1">
+    <row r="53" spans="1:1" ht="22.8" customHeight="1">
       <c r="A53" s="4"/>
     </row>
-    <row r="54" spans="1:1" ht="22.75" customHeight="1">
+    <row r="54" spans="1:1" ht="22.8" customHeight="1">
       <c r="A54" s="4"/>
     </row>
-    <row r="55" spans="1:1" ht="22.75" customHeight="1">
+    <row r="55" spans="1:1" ht="22.8" customHeight="1">
       <c r="A55" s="4"/>
     </row>
-    <row r="56" spans="1:1" ht="22.75" customHeight="1">
+    <row r="56" spans="1:1" ht="22.8" customHeight="1">
       <c r="A56" s="4"/>
     </row>
-    <row r="57" spans="1:1" ht="22.75" customHeight="1">
+    <row r="57" spans="1:1" ht="22.8" customHeight="1">
       <c r="A57" s="4"/>
     </row>
-    <row r="58" spans="1:1" ht="22.75" customHeight="1">
+    <row r="58" spans="1:1" ht="22.8" customHeight="1">
       <c r="A58" s="4"/>
     </row>
-    <row r="59" spans="1:1" ht="22.75" customHeight="1">
+    <row r="59" spans="1:1" ht="22.8" customHeight="1">
       <c r="A59" s="4"/>
     </row>
-    <row r="60" spans="1:1" ht="22.75" customHeight="1">
+    <row r="60" spans="1:1" ht="22.8" customHeight="1">
       <c r="A60" s="4"/>
     </row>
-    <row r="61" spans="1:1" ht="22.75" customHeight="1">
+    <row r="61" spans="1:1" ht="22.8" customHeight="1">
       <c r="A61" s="4"/>
     </row>
-    <row r="62" spans="1:1" ht="22.75" customHeight="1">
+    <row r="62" spans="1:1" ht="22.8" customHeight="1">
       <c r="A62" s="4"/>
     </row>
-    <row r="63" spans="1:1" ht="22.75" customHeight="1">
+    <row r="63" spans="1:1" ht="22.8" customHeight="1">
       <c r="A63" s="4"/>
     </row>
-    <row r="64" spans="1:1" ht="22.75" customHeight="1">
+    <row r="64" spans="1:1" ht="22.8" customHeight="1">
       <c r="A64" s="4"/>
     </row>
-    <row r="65" spans="1:1" ht="22.75" customHeight="1">
+    <row r="65" spans="1:1" ht="22.8" customHeight="1">
       <c r="A65" s="4"/>
     </row>
-    <row r="66" spans="1:1" ht="22.75" customHeight="1">
+    <row r="66" spans="1:1" ht="22.8" customHeight="1">
       <c r="A66" s="4"/>
     </row>
-    <row r="67" spans="1:1" ht="22.75" customHeight="1">
+    <row r="67" spans="1:1" ht="22.8" customHeight="1">
       <c r="A67" s="4"/>
     </row>
-    <row r="68" spans="1:1" ht="22.75" customHeight="1">
+    <row r="68" spans="1:1" ht="22.8" customHeight="1">
       <c r="A68" s="4"/>
     </row>
-    <row r="69" spans="1:1" ht="22.75" customHeight="1">
+    <row r="69" spans="1:1" ht="22.8" customHeight="1">
       <c r="A69" s="4"/>
     </row>
-    <row r="70" spans="1:1" ht="22.75" customHeight="1">
+    <row r="70" spans="1:1" ht="22.8" customHeight="1">
       <c r="A70" s="4"/>
     </row>
-    <row r="71" spans="1:1" ht="22.75" customHeight="1">
+    <row r="71" spans="1:1" ht="22.8" customHeight="1">
       <c r="A71" s="4"/>
     </row>
-    <row r="72" spans="1:1" ht="22.75" customHeight="1">
+    <row r="72" spans="1:1" ht="22.8" customHeight="1">
       <c r="A72" s="4"/>
     </row>
-    <row r="73" spans="1:1" ht="22.75" customHeight="1">
+    <row r="73" spans="1:1" ht="22.8" customHeight="1">
       <c r="A73" s="4"/>
     </row>
-    <row r="74" spans="1:1" ht="22.75" customHeight="1">
+    <row r="74" spans="1:1" ht="22.8" customHeight="1">
       <c r="A74" s="4"/>
     </row>
-    <row r="75" spans="1:1" ht="22.75" customHeight="1">
+    <row r="75" spans="1:1" ht="22.8" customHeight="1">
       <c r="A75" s="4"/>
     </row>
-    <row r="76" spans="1:1" ht="22.75" customHeight="1">
+    <row r="76" spans="1:1" ht="22.8" customHeight="1">
       <c r="A76" s="4"/>
     </row>
-    <row r="77" spans="1:1" ht="22.75" customHeight="1">
+    <row r="77" spans="1:1" ht="22.8" customHeight="1">
       <c r="A77" s="4"/>
     </row>
-    <row r="78" spans="1:1" ht="22.75" customHeight="1">
+    <row r="78" spans="1:1" ht="22.8" customHeight="1">
       <c r="A78" s="4"/>
     </row>
-    <row r="79" spans="1:1" ht="22.75" customHeight="1">
+    <row r="79" spans="1:1" ht="22.8" customHeight="1">
       <c r="A79" s="4"/>
     </row>
-    <row r="80" spans="1:1" ht="22.75" customHeight="1">
+    <row r="80" spans="1:1" ht="22.8" customHeight="1">
       <c r="A80" s="4"/>
     </row>
-    <row r="81" spans="1:1" ht="22.75" customHeight="1">
+    <row r="81" spans="1:1" ht="22.8" customHeight="1">
       <c r="A81" s="4"/>
     </row>
-    <row r="82" spans="1:1" ht="22.75" customHeight="1">
+    <row r="82" spans="1:1" ht="22.8" customHeight="1">
       <c r="A82" s="4"/>
     </row>
-    <row r="83" spans="1:1" ht="22.75" customHeight="1">
+    <row r="83" spans="1:1" ht="22.8" customHeight="1">
       <c r="A83" s="4"/>
     </row>
-    <row r="84" spans="1:1" ht="22.75" customHeight="1">
+    <row r="84" spans="1:1" ht="22.8" customHeight="1">
       <c r="A84" s="4"/>
     </row>
-    <row r="85" spans="1:1" ht="22.75" customHeight="1">
+    <row r="85" spans="1:1" ht="22.8" customHeight="1">
       <c r="A85" s="4"/>
     </row>
-    <row r="86" spans="1:1" ht="22.75" customHeight="1">
+    <row r="86" spans="1:1" ht="22.8" customHeight="1">
       <c r="A86" s="4"/>
     </row>
-    <row r="87" spans="1:1" ht="22.75" customHeight="1">
+    <row r="87" spans="1:1" ht="22.8" customHeight="1">
       <c r="A87" s="4"/>
     </row>
-    <row r="88" spans="1:1" ht="22.75" customHeight="1">
+    <row r="88" spans="1:1" ht="22.8" customHeight="1">
       <c r="A88" s="4"/>
     </row>
-    <row r="89" spans="1:1" ht="22.75" customHeight="1">
+    <row r="89" spans="1:1" ht="22.8" customHeight="1">
       <c r="A89" s="4"/>
     </row>
-    <row r="90" spans="1:1" ht="22.75" customHeight="1">
+    <row r="90" spans="1:1" ht="22.8" customHeight="1">
       <c r="A90" s="4"/>
     </row>
-    <row r="91" spans="1:1" ht="22.75" customHeight="1">
+    <row r="91" spans="1:1" ht="22.8" customHeight="1">
       <c r="A91" s="4"/>
     </row>
-    <row r="92" spans="1:1" ht="22.75" customHeight="1">
+    <row r="92" spans="1:1" ht="22.8" customHeight="1">
       <c r="A92" s="4"/>
     </row>
-    <row r="93" spans="1:1" ht="22.75" customHeight="1">
+    <row r="93" spans="1:1" ht="22.8" customHeight="1">
       <c r="A93" s="4"/>
     </row>
-    <row r="94" spans="1:1" ht="22.75" customHeight="1">
+    <row r="94" spans="1:1" ht="22.8" customHeight="1">
       <c r="A94" s="4"/>
     </row>
-    <row r="95" spans="1:1" ht="22.75" customHeight="1">
+    <row r="95" spans="1:1" ht="22.8" customHeight="1">
       <c r="A95" s="4"/>
     </row>
-    <row r="96" spans="1:1" ht="22.75" customHeight="1">
+    <row r="96" spans="1:1" ht="22.8" customHeight="1">
       <c r="A96" s="4"/>
     </row>
-    <row r="97" spans="1:1" ht="22.75" customHeight="1">
+    <row r="97" spans="1:1" ht="22.8" customHeight="1">
       <c r="A97" s="4"/>
     </row>
-    <row r="98" spans="1:1" ht="22.75" customHeight="1">
+    <row r="98" spans="1:1" ht="22.8" customHeight="1">
       <c r="A98" s="4"/>
     </row>
-    <row r="99" spans="1:1" ht="22.75" customHeight="1">
+    <row r="99" spans="1:1" ht="22.8" customHeight="1">
       <c r="A99" s="4"/>
     </row>
-    <row r="100" spans="1:1" ht="22.75" customHeight="1">
+    <row r="100" spans="1:1" ht="22.8" customHeight="1">
       <c r="A100" s="4"/>
     </row>
-    <row r="101" spans="1:1" ht="22.75" customHeight="1">
+    <row r="101" spans="1:1" ht="22.8" customHeight="1">
       <c r="A101" s="4"/>
     </row>
-    <row r="102" spans="1:1" ht="22.75" customHeight="1">
+    <row r="102" spans="1:1" ht="22.8" customHeight="1">
       <c r="A102" s="4"/>
     </row>
-    <row r="103" spans="1:1" ht="22.75" customHeight="1">
+    <row r="103" spans="1:1" ht="22.8" customHeight="1">
       <c r="A103" s="4"/>
     </row>
-    <row r="104" spans="1:1" ht="22.75" customHeight="1">
+    <row r="104" spans="1:1" ht="22.8" customHeight="1">
       <c r="A104" s="4"/>
     </row>
-    <row r="105" spans="1:1" ht="22.75" customHeight="1">
+    <row r="105" spans="1:1" ht="22.8" customHeight="1">
       <c r="A105" s="4"/>
     </row>
-    <row r="106" spans="1:1" ht="22.75" customHeight="1">
+    <row r="106" spans="1:1" ht="22.8" customHeight="1">
       <c r="A106" s="4"/>
     </row>
-    <row r="107" spans="1:1" ht="22.75" customHeight="1">
+    <row r="107" spans="1:1" ht="22.8" customHeight="1">
       <c r="A107" s="4"/>
     </row>
-    <row r="108" spans="1:1" ht="22.75" customHeight="1">
+    <row r="108" spans="1:1" ht="22.8" customHeight="1">
       <c r="A108" s="4"/>
     </row>
-    <row r="109" spans="1:1" ht="22.75" customHeight="1">
+    <row r="109" spans="1:1" ht="22.8" customHeight="1">
       <c r="A109" s="4"/>
     </row>
-    <row r="110" spans="1:1" ht="22.75" customHeight="1">
+    <row r="110" spans="1:1" ht="22.8" customHeight="1">
       <c r="A110" s="4"/>
     </row>
-    <row r="111" spans="1:1" ht="22.75" customHeight="1">
+    <row r="111" spans="1:1" ht="22.8" customHeight="1">
       <c r="A111" s="4"/>
     </row>
-    <row r="112" spans="1:1" ht="22.75" customHeight="1">
+    <row r="112" spans="1:1" ht="22.8" customHeight="1">
       <c r="A112" s="4"/>
     </row>
-    <row r="113" spans="1:1" ht="22.75" customHeight="1">
+    <row r="113" spans="1:1" ht="22.8" customHeight="1">
       <c r="A113" s="4"/>
     </row>
-    <row r="114" spans="1:1" ht="22.75" customHeight="1">
+    <row r="114" spans="1:1" ht="22.8" customHeight="1">
       <c r="A114" s="4"/>
     </row>
-    <row r="115" spans="1:1" ht="22.75" customHeight="1">
+    <row r="115" spans="1:1" ht="22.8" customHeight="1">
       <c r="A115" s="4"/>
     </row>
-    <row r="116" spans="1:1" ht="22.75" customHeight="1">
+    <row r="116" spans="1:1" ht="22.8" customHeight="1">
       <c r="A116" s="4"/>
     </row>
-    <row r="117" spans="1:1" ht="22.75" customHeight="1">
+    <row r="117" spans="1:1" ht="22.8" customHeight="1">
       <c r="A117" s="4"/>
     </row>
-    <row r="118" spans="1:1" ht="22.75" customHeight="1">
+    <row r="118" spans="1:1" ht="22.8" customHeight="1">
       <c r="A118" s="4"/>
     </row>
-    <row r="119" spans="1:1" ht="22.75" customHeight="1">
+    <row r="119" spans="1:1" ht="22.8" customHeight="1">
       <c r="A119" s="4"/>
     </row>
-    <row r="120" spans="1:1" ht="22.75" customHeight="1">
+    <row r="120" spans="1:1" ht="22.8" customHeight="1">
       <c r="A120" s="4"/>
     </row>
-    <row r="121" spans="1:1" ht="22.75" customHeight="1">
+    <row r="121" spans="1:1" ht="22.8" customHeight="1">
       <c r="A121" s="4"/>
     </row>
-    <row r="122" spans="1:1" ht="22.75" customHeight="1">
+    <row r="122" spans="1:1" ht="22.8" customHeight="1">
       <c r="A122" s="4"/>
     </row>
-    <row r="123" spans="1:1" ht="22.75" customHeight="1">
+    <row r="123" spans="1:1" ht="22.8" customHeight="1">
       <c r="A123" s="4"/>
     </row>
-    <row r="124" spans="1:1" ht="22.75" customHeight="1">
+    <row r="124" spans="1:1" ht="22.8" customHeight="1">
       <c r="A124" s="4"/>
     </row>
-    <row r="125" spans="1:1" ht="22.75" customHeight="1">
+    <row r="125" spans="1:1" ht="22.8" customHeight="1">
       <c r="A125" s="4"/>
     </row>
-    <row r="126" spans="1:1" ht="22.75" customHeight="1">
+    <row r="126" spans="1:1" ht="22.8" customHeight="1">
       <c r="A126" s="4"/>
     </row>
-    <row r="127" spans="1:1" ht="22.75" customHeight="1">
+    <row r="127" spans="1:1" ht="22.8" customHeight="1">
       <c r="A127" s="4"/>
     </row>
-    <row r="128" spans="1:1" ht="22.75" customHeight="1">
+    <row r="128" spans="1:1" ht="22.8" customHeight="1">
       <c r="A128" s="4"/>
     </row>
-    <row r="129" spans="1:1" ht="22.75" customHeight="1">
+    <row r="129" spans="1:1" ht="22.8" customHeight="1">
       <c r="A129" s="4"/>
     </row>
-    <row r="130" spans="1:1" ht="22.75" customHeight="1">
+    <row r="130" spans="1:1" ht="22.8" customHeight="1">
       <c r="A130" s="4"/>
     </row>
-    <row r="131" spans="1:1" ht="22.75" customHeight="1">
+    <row r="131" spans="1:1" ht="22.8" customHeight="1">
       <c r="A131" s="4"/>
     </row>
-    <row r="132" spans="1:1" ht="22.75" customHeight="1">
+    <row r="132" spans="1:1" ht="22.8" customHeight="1">
       <c r="A132" s="4"/>
     </row>
-    <row r="133" spans="1:1" ht="22.75" customHeight="1">
+    <row r="133" spans="1:1" ht="22.8" customHeight="1">
       <c r="A133" s="4"/>
     </row>
-    <row r="134" spans="1:1" ht="22.75" customHeight="1">
+    <row r="134" spans="1:1" ht="22.8" customHeight="1">
       <c r="A134" s="4"/>
     </row>
-    <row r="135" spans="1:1" ht="22.75" customHeight="1">
+    <row r="135" spans="1:1" ht="22.8" customHeight="1">
       <c r="A135" s="4"/>
     </row>
-    <row r="136" spans="1:1" ht="22.75" customHeight="1">
+    <row r="136" spans="1:1" ht="22.8" customHeight="1">
       <c r="A136" s="4"/>
     </row>
-    <row r="137" spans="1:1" ht="22.75" customHeight="1">
+    <row r="137" spans="1:1" ht="22.8" customHeight="1">
       <c r="A137" s="4"/>
     </row>
-    <row r="138" spans="1:1" ht="22.75" customHeight="1">
+    <row r="138" spans="1:1" ht="22.8" customHeight="1">
       <c r="A138" s="4"/>
     </row>
-    <row r="139" spans="1:1" ht="22.75" customHeight="1">
+    <row r="139" spans="1:1" ht="22.8" customHeight="1">
       <c r="A139" s="4"/>
     </row>
-    <row r="140" spans="1:1" ht="22.75" customHeight="1">
+    <row r="140" spans="1:1" ht="22.8" customHeight="1">
       <c r="A140" s="4"/>
     </row>
-    <row r="141" spans="1:1" ht="22.75" customHeight="1">
+    <row r="141" spans="1:1" ht="22.8" customHeight="1">
       <c r="A141" s="4"/>
     </row>
-    <row r="142" spans="1:1" ht="22.75" customHeight="1">
+    <row r="142" spans="1:1" ht="22.8" customHeight="1">
       <c r="A142" s="4"/>
     </row>
-    <row r="143" spans="1:1" ht="22.75" customHeight="1">
+    <row r="143" spans="1:1" ht="22.8" customHeight="1">
       <c r="A143" s="4"/>
     </row>
-    <row r="144" spans="1:1" ht="22.75" customHeight="1">
+    <row r="144" spans="1:1" ht="22.8" customHeight="1">
       <c r="A144" s="4"/>
     </row>
-    <row r="145" spans="1:1" ht="22.75" customHeight="1">
+    <row r="145" spans="1:1" ht="22.8" customHeight="1">
       <c r="A145" s="4"/>
     </row>
-    <row r="146" spans="1:1" ht="22.75" customHeight="1">
+    <row r="146" spans="1:1" ht="22.8" customHeight="1">
       <c r="A146" s="4"/>
     </row>
-    <row r="147" spans="1:1" ht="22.75" customHeight="1">
+    <row r="147" spans="1:1" ht="22.8" customHeight="1">
       <c r="A147" s="4"/>
     </row>
-    <row r="148" spans="1:1" ht="22.75" customHeight="1">
+    <row r="148" spans="1:1" ht="22.8" customHeight="1">
       <c r="A148" s="4"/>
     </row>
-    <row r="149" spans="1:1" ht="22.75" customHeight="1">
+    <row r="149" spans="1:1" ht="22.8" customHeight="1">
       <c r="A149" s="4"/>
     </row>
-    <row r="150" spans="1:1" ht="22.75" customHeight="1">
+    <row r="150" spans="1:1" ht="22.8" customHeight="1">
       <c r="A150" s="4"/>
     </row>
-    <row r="151" spans="1:1" ht="22.75" customHeight="1">
+    <row r="151" spans="1:1" ht="22.8" customHeight="1">
       <c r="A151" s="4"/>
     </row>
-    <row r="152" spans="1:1" ht="22.75" customHeight="1">
+    <row r="152" spans="1:1" ht="22.8" customHeight="1">
       <c r="A152" s="4"/>
     </row>
-    <row r="153" spans="1:1" ht="22.75" customHeight="1">
+    <row r="153" spans="1:1" ht="22.8" customHeight="1">
       <c r="A153" s="4"/>
     </row>
-    <row r="154" spans="1:1" ht="22.75" customHeight="1">
+    <row r="154" spans="1:1" ht="22.8" customHeight="1">
       <c r="A154" s="4"/>
     </row>
-    <row r="155" spans="1:1" ht="22.75" customHeight="1">
+    <row r="155" spans="1:1" ht="22.8" customHeight="1">
       <c r="A155" s="4"/>
     </row>
-    <row r="156" spans="1:1" ht="22.75" customHeight="1">
+    <row r="156" spans="1:1" ht="22.8" customHeight="1">
       <c r="A156" s="4"/>
     </row>
-    <row r="157" spans="1:1" ht="22.75" customHeight="1">
+    <row r="157" spans="1:1" ht="22.8" customHeight="1">
       <c r="A157" s="4"/>
     </row>
-    <row r="158" spans="1:1" ht="22.75" customHeight="1">
+    <row r="158" spans="1:1" ht="22.8" customHeight="1">
       <c r="A158" s="4"/>
     </row>
-    <row r="159" spans="1:1" ht="22.75" customHeight="1">
+    <row r="159" spans="1:1" ht="22.8" customHeight="1">
       <c r="A159" s="4"/>
     </row>
-    <row r="160" spans="1:1" ht="22.75" customHeight="1">
+    <row r="160" spans="1:1" ht="22.8" customHeight="1">
       <c r="A160" s="4"/>
     </row>
-    <row r="161" spans="1:1" ht="22.75" customHeight="1">
+    <row r="161" spans="1:1" ht="22.8" customHeight="1">
       <c r="A161" s="4"/>
     </row>
-    <row r="162" spans="1:1" ht="22.75" customHeight="1">
+    <row r="162" spans="1:1" ht="22.8" customHeight="1">
       <c r="A162" s="4"/>
     </row>
-    <row r="163" spans="1:1" ht="22.75" customHeight="1">
+    <row r="163" spans="1:1" ht="22.8" customHeight="1">
       <c r="A163" s="4"/>
     </row>
-    <row r="164" spans="1:1" ht="22.75" customHeight="1">
+    <row r="164" spans="1:1" ht="22.8" customHeight="1">
       <c r="A164" s="4"/>
     </row>
-    <row r="165" spans="1:1" ht="22.75" customHeight="1">
+    <row r="165" spans="1:1" ht="22.8" customHeight="1">
       <c r="A165" s="4"/>
     </row>
-    <row r="166" spans="1:1" ht="22.75" customHeight="1">
+    <row r="166" spans="1:1" ht="22.8" customHeight="1">
       <c r="A166" s="4"/>
     </row>
-    <row r="167" spans="1:1" ht="22.75" customHeight="1">
+    <row r="167" spans="1:1" ht="22.8" customHeight="1">
       <c r="A167" s="4"/>
     </row>
-    <row r="168" spans="1:1" ht="22.75" customHeight="1">
+    <row r="168" spans="1:1" ht="22.8" customHeight="1">
       <c r="A168" s="4"/>
     </row>
-    <row r="169" spans="1:1" ht="22.75" customHeight="1">
+    <row r="169" spans="1:1" ht="22.8" customHeight="1">
       <c r="A169" s="4"/>
     </row>
-    <row r="170" spans="1:1" ht="22.75" customHeight="1">
+    <row r="170" spans="1:1" ht="22.8" customHeight="1">
       <c r="A170" s="4"/>
     </row>
-    <row r="171" spans="1:1" ht="22.75" customHeight="1">
+    <row r="171" spans="1:1" ht="22.8" customHeight="1">
       <c r="A171" s="4"/>
     </row>
-    <row r="172" spans="1:1" ht="22.75" customHeight="1">
+    <row r="172" spans="1:1" ht="22.8" customHeight="1">
       <c r="A172" s="4"/>
     </row>
-    <row r="173" spans="1:1" ht="22.75" customHeight="1">
+    <row r="173" spans="1:1" ht="22.8" customHeight="1">
       <c r="A173" s="4"/>
     </row>
-    <row r="174" spans="1:1" ht="22.75" customHeight="1">
+    <row r="174" spans="1:1" ht="22.8" customHeight="1">
       <c r="A174" s="4"/>
     </row>
-    <row r="175" spans="1:1" ht="22.75" customHeight="1">
+    <row r="175" spans="1:1" ht="22.8" customHeight="1">
       <c r="A175" s="4"/>
     </row>
-    <row r="176" spans="1:1" ht="22.75" customHeight="1">
+    <row r="176" spans="1:1" ht="22.8" customHeight="1">
       <c r="A176" s="4"/>
     </row>
-    <row r="177" spans="1:1" ht="22.75" customHeight="1">
+    <row r="177" spans="1:1" ht="22.8" customHeight="1">
       <c r="A177" s="4"/>
     </row>
-    <row r="178" spans="1:1" ht="22.75" customHeight="1">
+    <row r="178" spans="1:1" ht="22.8" customHeight="1">
       <c r="A178" s="4"/>
     </row>
-    <row r="179" spans="1:1" ht="22.75" customHeight="1">
+    <row r="179" spans="1:1" ht="22.8" customHeight="1">
       <c r="A179" s="4"/>
     </row>
-    <row r="180" spans="1:1" ht="22.75" customHeight="1">
+    <row r="180" spans="1:1" ht="22.8" customHeight="1">
       <c r="A180" s="4"/>
     </row>
-    <row r="181" spans="1:1" ht="22.75" customHeight="1">
+    <row r="181" spans="1:1" ht="22.8" customHeight="1">
       <c r="A181" s="4"/>
     </row>
-    <row r="182" spans="1:1" ht="22.75" customHeight="1">
+    <row r="182" spans="1:1" ht="22.8" customHeight="1">
       <c r="A182" s="4"/>
     </row>
-    <row r="183" spans="1:1" ht="22.75" customHeight="1">
+    <row r="183" spans="1:1" ht="22.8" customHeight="1">
       <c r="A183" s="4"/>
     </row>
-    <row r="184" spans="1:1" ht="22.75" customHeight="1">
+    <row r="184" spans="1:1" ht="22.8" customHeight="1">
       <c r="A184" s="4"/>
     </row>
-    <row r="185" spans="1:1" ht="22.75" customHeight="1">
+    <row r="185" spans="1:1" ht="22.8" customHeight="1">
       <c r="A185" s="4"/>
     </row>
-    <row r="186" spans="1:1" ht="22.75" customHeight="1">
+    <row r="186" spans="1:1" ht="22.8" customHeight="1">
       <c r="A186" s="4"/>
     </row>
-    <row r="187" spans="1:1" ht="22.75" customHeight="1">
+    <row r="187" spans="1:1" ht="22.8" customHeight="1">
       <c r="A187" s="4"/>
     </row>
-    <row r="188" spans="1:1" ht="22.75" customHeight="1">
+    <row r="188" spans="1:1" ht="22.8" customHeight="1">
       <c r="A188" s="4"/>
+    </row>
+    <row r="189" spans="1:1" ht="22.8" customHeight="1">
+      <c r="A189" s="4"/>
+    </row>
+    <row r="190" spans="1:1" ht="22.8" customHeight="1">
+      <c r="A190" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125978" footer="0.31496062992125978"/>
@@ -1972,18 +2137,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B3:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.90625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.90625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="41.36328125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="42.453125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="43.90625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="38.08984375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="43.6328125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.90625" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="10.90625" style="1"/>
+    <col min="1" max="1" width="10.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="41.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="42.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="43.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="38.109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="43.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.88671875" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:2">

</xml_diff>